<commit_message>
Advanced AI Demand Forecasting Platform
</commit_message>
<xml_diff>
--- a/Backend/forecast_report.xlsx
+++ b/Backend/forecast_report.xlsx
@@ -415,13 +415,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>future_day</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -433,101 +433,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Day 1</t>
+          <t>2025-07-20</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12442.34</v>
+        <v>152875.9125</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Day 2</t>
+          <t>2025-07-21</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12402.63</v>
+        <v>76488.59999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Day 3</t>
+          <t>2025-07-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12362.91</v>
+        <v>103866.0875</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Day 4</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12323.2</v>
+        <v>113680.9125</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Day 5</t>
+          <t>2025-07-24</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12283.49</v>
+        <v>77152.78750000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Day 6</t>
+          <t>2025-07-25</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12243.77</v>
+        <v>78757.625</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Day 7</t>
+          <t>2025-07-26</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12204.06</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Day 8</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>12164.35</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Day 9</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>12124.64</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Day 10</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>12084.92</v>
+        <v>121537.05</v>
       </c>
     </row>
   </sheetData>
@@ -541,13 +511,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>future_day</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -559,101 +529,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Day 1</t>
+          <t>2025-07-20</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>103.69</v>
+        <v>122300.73</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Day 2</t>
+          <t>2025-07-21</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>103.36</v>
+        <v>61190.88</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Day 3</t>
+          <t>2025-07-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>103.02</v>
+        <v>83092.87</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Day 4</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>102.69</v>
+        <v>90944.73</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Day 5</t>
+          <t>2025-07-24</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>102.36</v>
+        <v>61722.23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Day 6</t>
+          <t>2025-07-25</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>102.03</v>
+        <v>63006.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Day 7</t>
+          <t>2025-07-26</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>101.7</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Day 8</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>101.37</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Day 9</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>101.04</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Day 10</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>100.71</v>
+        <v>97229.64</v>
       </c>
     </row>
   </sheetData>
@@ -667,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -685,101 +625,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Electronic Accessories</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>535</v>
+        <v>54321</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Food and Beverages</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>415</v>
+        <v>48211</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tablet</t>
+          <t>Fashion Accessories</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Printer</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Speaker</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Smartwatch</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Headphones</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Keyboard</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>123</v>
+        <v>45990</v>
       </c>
     </row>
   </sheetData>

</xml_diff>